<commit_message>
Update building_data.json: Adjust generated_at timestamp and refine source_notes for church model
</commit_message>
<xml_diff>
--- a/output/block147_building_data.xlsx
+++ b/output/block147_building_data.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12 00:51</t>
+          <t>2026-05-12 00:54</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>special church roof: low tile body, shallow low kubbe with 3 glazed marks; kubbe centered at (670342.95, 4539707.85) from Pervititch GeoTIFF kubbe mark; clocher 16.9 m from Pervititch raster clocher square within W-39/1</t>
+          <t>special church roof: low tile body, curved lead/zinc kubbe with 3 arched glazed eyes; kubbe centered at (670342.95, 4539707.85) from Pervititch GeoTIFF kubbe mark; clocher 16.9 m from Pervititch raster clocher square within W-39/1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Block 147 Viewer and Presentation Assets
- Updated the redirect URL in index.html and viewer.html to reflect the new build version (20260512-0122).
- Added a new README.md file in the presentation directory detailing the visual assets for Block 147.
- Included various image assets for the presentation, including church images, flow diagrams, and maps.
- Adjusted geometry manifest and LOD3 coverage reports to reflect updated building dimensions.
- Enhanced the building geometry builder and church builder scripts to improve window placements and dimensions.
</commit_message>
<xml_diff>
--- a/output/block147_building_data.xlsx
+++ b/output/block147_building_data.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12 00:54</t>
+          <t>2026-05-12 01:22</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>ChurchBody, ChurchDome, Clocher, CorniceSurface, Door, GroundSurface, HeaderSurface, JambSurface, Mullion, PlinthSurface, RoofSurface, SillSurface, StringcourseSurface, Window</t>
+          <t>ChurchBody, ChurchDome, Clocher, CorniceSurface, GroundSurface, HeaderSurface, JambSurface, Mullion, PlinthSurface, RoofSurface, SillSurface, StringcourseSurface, Window</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update geometry manifest and reports for W-39/2 entrance adjustments
- Adjusted dimensions and attributes for W-39/2 in geometry_manifest.md
- Updated coverage data for W-39/1.camli_vitre_passage in lod3_coverage.md
- Modified opening audit details for W-39/2 to reflect accurate mapping evidence
- Implemented new geometry for W-39/2 entrance in building_geometry_builder.py, ensuring door is mounted flush to the existing stone wall with detailed jamb and trim features
</commit_message>
<xml_diff>
--- a/output/block147_building_data.xlsx
+++ b/output/block147_building_data.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12 02:14</t>
+          <t>2026-05-12 02:24</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5582,7 @@
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>map+photo:cesme-left-side-adjacent-door: 1</t>
+          <t>map:pervititch:39-2-entrance-mounted-to-wall: 1</t>
         </is>
       </c>
     </row>
@@ -11004,7 +11004,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>map+photo:cesme-left-side-adjacent-door: 1</t>
+          <t>map:pervititch:39-2-entrance-mounted-to-wall: 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update viewer and reports for Block 147
- Updated the refresh URL in index.html and viewer.html to version 20260512-0247.
- Modified geometry_manifest.md to correct dimensions for W-39/2 and W-39-1.camli_vitre_passage.
- Adjusted lod3_coverage.md to reflect changes in coverage for W-39/2 and W-39-1.camli_vitre_passage.
- Revised opening_audit.md to update the status of W-39/2 and W-39-1.camli_vitre_passage.
- Implemented a new entrance placement for W-39/2 in render_manual.py.
- Removed deprecated entrance geometry for W-39/2 in building_geometry_builder.py and updated metadata accordingly.
</commit_message>
<xml_diff>
--- a/output/block147_building_data.xlsx
+++ b/output/block147_building_data.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12 02:31</t>
+          <t>2026-05-12 02:46</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
         </is>
       </c>
       <c r="V34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W34" s="2" t="n">
         <v>0</v>
@@ -5557,7 +5557,7 @@
         </is>
       </c>
       <c r="V37" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W37" s="2" t="n">
         <v>0</v>
@@ -5577,12 +5577,12 @@
       </c>
       <c r="AA37" s="2" t="inlineStr">
         <is>
-          <t>Door, GroundSurface, MonumentBody, RoofSurface</t>
+          <t>GroundSurface, MonumentBody, RoofSurface</t>
         </is>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>map:pervititch:39-2-entrance-mounted-to-wall: 1</t>
+          <t>non-building asset</t>
         </is>
       </c>
     </row>
@@ -11004,7 +11004,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>map:pervititch:39-2-entrance-mounted-to-wall: 1</t>
+          <t>non-building asset</t>
         </is>
       </c>
     </row>

</xml_diff>